<commit_message>
DATA. Nueva construccion y reentrenamiento de modelos para ENG
</commit_message>
<xml_diff>
--- a/data/england/p3_data_preparation/df_hiper_prep.xlsx
+++ b/data/england/p3_data_preparation/df_hiper_prep.xlsx
@@ -471,8 +471,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>30</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[30, 180]</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>3</v>
@@ -481,14 +483,14 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DATA. Reentrenamiento de modelos para todos los paises incluyendo redes neuronales, nuevo fifa 25, eliminando partidos antes de 2012, mejora de integracion, etc.
</commit_message>
<xml_diff>
--- a/data/england/p3_data_preparation/df_hiper_prep.xlsx
+++ b/data/england/p3_data_preparation/df_hiper_prep.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,25 +446,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>dif_con_against</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>thr_corr</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>thr_fs</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fill_na</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_years_to_select</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>comp_to_select</t>
         </is>
@@ -473,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[90]</t>
+          <t>[30, 180]</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -482,17 +487,20 @@
       <c r="C2" t="b">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
-        <v>0.9</v>
+      <c r="D2" t="b">
+        <v>0</v>
       </c>
       <c r="E2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.5</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
         <v>3</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>[481, 482, 483, 484]</t>
         </is>

</xml_diff>